<commit_message>
Fees & Discounts: resolve FD-FIN duplicate IDs (group-B document cases → FD-DOC-*), rebuild workbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
+++ b/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
@@ -8633,7 +8633,7 @@
     <row r="111">
       <c r="A111" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-001</t>
+          <t>FD-DOC-001</t>
         </is>
       </c>
       <c r="B111" s="18" t="inlineStr">
@@ -8702,7 +8702,7 @@
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-002</t>
+          <t>FD-DOC-002</t>
         </is>
       </c>
       <c r="B112" s="15" t="inlineStr">
@@ -8768,7 +8768,7 @@
     <row r="113">
       <c r="A113" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-003</t>
+          <t>FD-DOC-003</t>
         </is>
       </c>
       <c r="B113" s="18" t="inlineStr">
@@ -8833,7 +8833,7 @@
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-004</t>
+          <t>FD-DOC-004</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
@@ -8903,7 +8903,7 @@
     <row r="115">
       <c r="A115" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-005</t>
+          <t>FD-DOC-005</t>
         </is>
       </c>
       <c r="B115" s="18" t="inlineStr">
@@ -8969,7 +8969,7 @@
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-006</t>
+          <t>FD-DOC-006</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
@@ -9038,7 +9038,7 @@
     <row r="117">
       <c r="A117" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-007</t>
+          <t>FD-DOC-007</t>
         </is>
       </c>
       <c r="B117" s="18" t="inlineStr">
@@ -9101,7 +9101,7 @@
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-008</t>
+          <t>FD-DOC-008</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="119">
       <c r="A119" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-009</t>
+          <t>FD-DOC-009</t>
         </is>
       </c>
       <c r="B119" s="18" t="inlineStr">
@@ -9231,7 +9231,7 @@
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-010</t>
+          <t>FD-DOC-010</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -9296,7 +9296,7 @@
     <row r="121">
       <c r="A121" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-011</t>
+          <t>FD-DOC-011</t>
         </is>
       </c>
       <c r="B121" s="18" t="inlineStr">
@@ -16676,7 +16676,7 @@
     <row r="112">
       <c r="A112" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-001</t>
+          <t>FD-DOC-001</t>
         </is>
       </c>
       <c r="B112" s="18" t="inlineStr">
@@ -16702,7 +16702,7 @@
     <row r="113">
       <c r="A113" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-002</t>
+          <t>FD-DOC-002</t>
         </is>
       </c>
       <c r="B113" s="15" t="inlineStr">
@@ -16728,7 +16728,7 @@
     <row r="114">
       <c r="A114" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-003</t>
+          <t>FD-DOC-003</t>
         </is>
       </c>
       <c r="B114" s="18" t="inlineStr">
@@ -16754,7 +16754,7 @@
     <row r="115">
       <c r="A115" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-004</t>
+          <t>FD-DOC-004</t>
         </is>
       </c>
       <c r="B115" s="15" t="inlineStr">
@@ -16780,7 +16780,7 @@
     <row r="116">
       <c r="A116" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-005</t>
+          <t>FD-DOC-005</t>
         </is>
       </c>
       <c r="B116" s="18" t="inlineStr">
@@ -16806,7 +16806,7 @@
     <row r="117">
       <c r="A117" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-006</t>
+          <t>FD-DOC-006</t>
         </is>
       </c>
       <c r="B117" s="15" t="inlineStr">
@@ -16832,7 +16832,7 @@
     <row r="118">
       <c r="A118" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-007</t>
+          <t>FD-DOC-007</t>
         </is>
       </c>
       <c r="B118" s="18" t="inlineStr">
@@ -16858,7 +16858,7 @@
     <row r="119">
       <c r="A119" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-008</t>
+          <t>FD-DOC-008</t>
         </is>
       </c>
       <c r="B119" s="15" t="inlineStr">
@@ -16884,7 +16884,7 @@
     <row r="120">
       <c r="A120" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-009</t>
+          <t>FD-DOC-009</t>
         </is>
       </c>
       <c r="B120" s="18" t="inlineStr">
@@ -16910,7 +16910,7 @@
     <row r="121">
       <c r="A121" s="14" t="inlineStr">
         <is>
-          <t>FD-FIN-010</t>
+          <t>FD-DOC-010</t>
         </is>
       </c>
       <c r="B121" s="15" t="inlineStr">
@@ -16936,7 +16936,7 @@
     <row r="122">
       <c r="A122" s="17" t="inlineStr">
         <is>
-          <t>FD-FIN-011</t>
+          <t>FD-DOC-011</t>
         </is>
       </c>
       <c r="B122" s="18" t="inlineStr">
@@ -19134,7 +19134,7 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>FD-FIN-001 (Group B), FD-TMPL-001, FD-EDIT-001</t>
+          <t>FD-DOC-001 (Group B), FD-TMPL-001, FD-EDIT-001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fees & Discounts: remove 'feature flag ON' precondition from all cases; renumber; regenerate CSV+workbook
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
+++ b/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
@@ -1011,10 +1011,9 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>1. The Fees &amp; Discounts feature flag is ON for the organization.
-2. You are logged in as a role that has Work Orders: Create &amp; Edit and See Financial Data.
-3. An open (not Invoiced, not Paid) work order exists; you are viewing it and are NOT in history mode.
-4. You are on the work order's Lines tab.</t>
+          <t>1. You are logged in as a role that has Work Orders: Create &amp; Edit and See Financial Data.
+2. An open (not Invoiced, not Paid) work order exists; you are viewing it and are NOT in history mode.
+3. You are on the work order's Lines tab.</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
@@ -1085,7 +1084,7 @@
       </c>
       <c r="H3" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order with subtotal exactly $10,715.39 (or any known subtotal) is open on the Lines tab.</t>
         </is>
       </c>
@@ -1163,7 +1162,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order with Work Order Total = $10,715.39 is open.</t>
         </is>
       </c>
@@ -1239,7 +1238,7 @@
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order is open; the location's template library contains 'Fleet Standard Discount (−10%)'.</t>
         </is>
       </c>
@@ -1315,7 +1314,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order is open with the Add dialog freshly opened (all fields blank).</t>
         </is>
       </c>
@@ -1393,7 +1392,7 @@
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order whose relevant base for the fee is exactly $100.00 is open.</t>
         </is>
       </c>
@@ -1466,7 +1465,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
@@ -1536,7 +1535,7 @@
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
@@ -1607,7 +1606,7 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. The whole-WO Add dialog is open with Name, Type='Fee', Calc type='Flat amount' set.</t>
         </is>
       </c>
@@ -1677,7 +1676,7 @@
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
@@ -1747,7 +1746,7 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order with Net Labor total $200.00, Net Parts total $100.00, Shop Supplies $0.00 (so Subtotal = $300.00), no other adjustments.</t>
         </is>
       </c>
@@ -1820,7 +1819,7 @@
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. A work order in Invoiced (or Paid) status is open.</t>
         </is>
       </c>
@@ -1891,9 +1890,8 @@
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Logged in as a role that HAS See Financial Data but does NOT have Work Orders: Create &amp; Edit.
-3. An open work order is open.</t>
+          <t>1. Logged in as a role that HAS See Financial Data but does NOT have Work Orders: Create &amp; Edit.
+2. An open work order is open.</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
@@ -1961,7 +1959,7 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. The whole-WO Add dialog is freshly open.</t>
         </is>
       </c>
@@ -2031,7 +2029,7 @@
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
@@ -2101,7 +2099,7 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit and See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit and See Financial Data.
 2. An open work order with a labor line, e.g. Line 1 'Service - Perform LOF and inspection', is open on the Lines tab.</t>
         </is>
       </c>
@@ -2173,7 +2171,7 @@
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a labor line whose gross labor price is exactly $150.00, no existing adjustments on that line.</t>
         </is>
       </c>
@@ -2247,7 +2245,7 @@
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with two or more labor lines is open on the Lines tab.</t>
         </is>
       </c>
@@ -2317,7 +2315,7 @@
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a labor line (any quantity/hours) is open.</t>
         </is>
       </c>
@@ -2388,7 +2386,7 @@
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a labor line that carries a 10% fee adjustment resolving to a non-zero amount.</t>
         </is>
       </c>
@@ -2460,7 +2458,7 @@
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a labor line that carries at least one fee/discount adjustment.</t>
         </is>
       </c>
@@ -2531,9 +2529,8 @@
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Logged in as a role with See Financial Data but WITHOUT Work Order Lines: Create &amp; Edit.
-3. An open work order with a labor line is open.</t>
+          <t>1. Logged in as a role with See Financial Data but WITHOUT Work Order Lines: Create &amp; Edit.
+2. An open work order with a labor line is open.</t>
         </is>
       </c>
       <c r="I23" s="18" t="inlineStr">
@@ -2602,7 +2599,7 @@
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part, e.g. '(LF3620) Engine Oil Filter', is open on the Lines or Parts tab.</t>
         </is>
       </c>
@@ -2674,7 +2671,7 @@
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part of quantity 3.</t>
         </is>
       </c>
@@ -2747,7 +2744,7 @@
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a requested (pending / not yet picked) part of quantity 2 at sell price $20.00 each.</t>
         </is>
       </c>
@@ -2820,7 +2817,7 @@
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part of quantity 3 at sell price $20.00 each (gross part total $60.00).</t>
         </is>
       </c>
@@ -2892,7 +2889,7 @@
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a requested part that already carries a % of Parts Total discount.</t>
         </is>
       </c>
@@ -2963,7 +2960,7 @@
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part carrying a discount that resolves to a non-zero amount.</t>
         </is>
       </c>
@@ -3035,7 +3032,7 @@
       </c>
       <c r="H30" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part that carries at least one adjustment.</t>
         </is>
       </c>
@@ -3106,7 +3103,7 @@
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part of quantity 1.</t>
         </is>
       </c>
@@ -3177,7 +3174,7 @@
       </c>
       <c r="H32" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order where Line 1 labor carries a 'Line discount' of −5% resolving to −$26.08.</t>
         </is>
       </c>
@@ -3248,7 +3245,7 @@
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order where part '(LF3620) Engine Oil Filter' carries a 'Parts Handling Fee' of +$3.75.</t>
         </is>
       </c>
@@ -3319,7 +3316,7 @@
       </c>
       <c r="H34" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order where the LF3620 part carries three adjustments: Part discount (−10%), Fleet discount (−5%), Parts Handling Fee (+$3.75).</t>
         </is>
       </c>
@@ -3393,7 +3390,7 @@
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order where the LF3620 part has base total $58.47 plus adjustments −$6.49, −$2.92, +$3.75.</t>
         </is>
       </c>
@@ -3464,7 +3461,7 @@
       </c>
       <c r="H36" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with at least one inline line-level adjustment.</t>
         </is>
       </c>
@@ -3535,7 +3532,7 @@
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order with 5 adjustments across scopes is open.</t>
         </is>
       </c>
@@ -3607,7 +3604,7 @@
       </c>
       <c r="H38" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order (e.g. S2-13274) with a whole-WO discount and line-level part/labor adjustments.</t>
         </is>
       </c>
@@ -3679,7 +3676,7 @@
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order with adjustments: Work order discount −$857.23, Part discount −$649.00, Fleet discount −$292.00, Parts Handling Fee +$3.75, Line discount −$260.77.</t>
         </is>
       </c>
@@ -3750,7 +3747,7 @@
       </c>
       <c r="H40" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order to which you add three adjustments in a known order: (a) Adjustment A first, (b) Adjustment B second, (c) Adjustment C third.</t>
         </is>
       </c>
@@ -3820,7 +3817,7 @@
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order with zero fee/discount adjustments of any scope.</t>
         </is>
       </c>
@@ -3889,7 +3886,7 @@
       </c>
       <c r="H42" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order with 5 adjustments (any scopes) netting to −$2,055.25.</t>
         </is>
       </c>
@@ -3961,7 +3958,7 @@
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. An open work order with 5 adjustments as in FD-FIN-001.</t>
         </is>
       </c>
@@ -4032,9 +4029,8 @@
       </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Variant (a): logged in with See Financial Data, an open WO with zero adjustments.
-3. Variant (b): logged in as a role WITHOUT See Financial Data, an open WO with adjustments.</t>
+          <t>1. Variant (a): logged in with See Financial Data, an open WO with zero adjustments.
+2. Variant (b): logged in as a role WITHOUT See Financial Data, an open WO with adjustments.</t>
         </is>
       </c>
       <c r="I44" s="15" t="inlineStr">
@@ -4103,7 +4099,7 @@
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data and Work Orders: Create &amp; Edit.
+          <t>1. Logged in with See Financial Data and Work Orders: Create &amp; Edit.
 2. An open work order with a whole-WO 'Early Payment Discount' of −8% resolving to −$857.23, plus some line-level adjustments.</t>
         </is>
       </c>
@@ -4175,7 +4171,7 @@
       </c>
       <c r="H46" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data + Work Orders: Create &amp; Edit.
+          <t>1. Logged in with See Financial Data + Work Orders: Create &amp; Edit.
 2. Variant (a): an open WO with only line-level adjustments and NO whole-WO adjustments.
 3. Variant (b): an open WO with at least one whole-WO adjustment.</t>
         </is>
@@ -4246,7 +4242,7 @@
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. A Parts page / WO parts view is open with part '#37346 Mobil 1 5W20' carrying exactly one adjustment 'Military Discount' −10%.</t>
         </is>
       </c>
@@ -4316,7 +4312,7 @@
       </c>
       <c r="H48" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. Parts page open with part '#55073 Mobil 1 5W20' carrying three adjustments (first = 'Parts Handling Fee' 2%).</t>
         </is>
       </c>
@@ -4386,7 +4382,7 @@
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data and the relevant change permission.
+          <t>1. Logged in with See Financial Data and the relevant change permission.
 2. Parts page open with part '#28439 Fleetguard FF5421' carrying no adjustments, on an editable sale/WO.</t>
         </is>
       </c>
@@ -4457,7 +4453,7 @@
       </c>
       <c r="H50" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. Parts page open with part '#55073 Mobil 1 5W20' carrying three adjustments (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).</t>
         </is>
       </c>
@@ -4530,7 +4526,7 @@
       </c>
       <c r="H51" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. The #55073 breakdown modal from FD-PCOL-004 is open (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).</t>
         </is>
       </c>
@@ -4598,7 +4594,7 @@
       </c>
       <c r="H52" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with the relevant change permission + See Financial Data.
+          <t>1. Logged in with the relevant change permission + See Financial Data.
 2. Parts page open with part #37346 carrying exactly ONE adjustment; the editable breakdown modal is open.</t>
         </is>
       </c>
@@ -4670,7 +4666,7 @@
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with See Financial Data.
+          <t>1. Logged in with See Financial Data.
 2. Parts page open for an Invoiced/Paid (non-editable) sale/WO with a part that has no adjustments.</t>
         </is>
       </c>
@@ -4740,7 +4736,7 @@
       </c>
       <c r="H54" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with the relevant change permission + See Financial Data.
+          <t>1. Logged in with the relevant change permission + See Financial Data.
 2. An open work order with an existing whole-WO percentage discount adjustment.</t>
         </is>
       </c>
@@ -4814,7 +4810,7 @@
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with the relevant change permission + See Financial Data.
+          <t>1. Logged in with the relevant change permission + See Financial Data.
 2. An open work order with an existing percentage adjustment whose base total has since changed (e.g. a line was added).</t>
         </is>
       </c>
@@ -4888,7 +4884,7 @@
       </c>
       <c r="H56" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with the relevant change permission + See Financial Data.
+          <t>1. Logged in with the relevant change permission + See Financial Data.
 2. An open work order with an existing adjustment; a condition that forces a save failure can be simulated (e.g. server error).</t>
         </is>
       </c>
@@ -4959,7 +4955,7 @@
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order with a whole-WO discount named 'Early Payment Discount'.</t>
         </is>
       </c>
@@ -5032,9 +5028,8 @@
       </c>
       <c r="H58" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Logged in as a role that HAS Work Orders: Create &amp; Edit and See Financial Data but does NOT have the separate 'Delete' permission.
-3. An open work order with a whole-WO adjustment.</t>
+          <t>1. Logged in as a role that HAS Work Orders: Create &amp; Edit and See Financial Data but does NOT have the separate 'Delete' permission.
+2. An open work order with a whole-WO adjustment.</t>
         </is>
       </c>
       <c r="I58" s="15" t="inlineStr">
@@ -5105,7 +5100,7 @@
       </c>
       <c r="H59" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order where a part carries a 'Fleet discount' adjustment shown inline.</t>
         </is>
       </c>
@@ -5178,7 +5173,7 @@
       </c>
       <c r="H60" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
 2. An open work order with a part of gross part total exactly $100.00.</t>
         </is>
       </c>
@@ -5253,7 +5248,7 @@
       </c>
       <c r="H61" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit, Work Order Lines: Create &amp; Edit, and See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit, Work Order Lines: Create &amp; Edit, and See Financial Data.
 2. An open work order with Gross Labor $200.00 and Gross Parts $100.00, no shop supplies.
 3. A Labor Line 10% discount already applied (Step 1: −$20.00, so Net Labor = $180.00).</t>
         </is>
@@ -5327,7 +5322,7 @@
       </c>
       <c r="H62" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON; logged in with Work Orders: Create &amp; Edit + See Financial Data.
+          <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
 2. An open work order; the location library has a 'Parts Handling Fee' template.</t>
         </is>
       </c>
@@ -5398,9 +5393,8 @@
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
-          <t>1. The Fees &amp; Discounts feature flag is ON for the organization.
-2. A test customer named ZZAUTOTEST Customer exists with exactly 2 default fees/discounts linked.
-3. You are logged in with Customer Management: Create &amp; Edit and Manage AP/AR permissions.</t>
+          <t>1. A test customer named ZZAUTOTEST Customer exists with exactly 2 default fees/discounts linked.
+2. You are logged in with Customer Management: Create &amp; Edit and Manage AP/AR permissions.</t>
         </is>
       </c>
       <c r="I63" s="18" t="inlineStr">
@@ -5470,7 +5464,7 @@
       </c>
       <c r="H64" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a customer with at least 1 default fee/discount exists.
+          <t>1. A customer with at least 1 default fee/discount exists.
 2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
@@ -5543,7 +5537,7 @@
       </c>
       <c r="H65" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a location template named "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%) exists and is NOT yet linked to the test customer.
+          <t>1. A location template named "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%) exists and is NOT yet linked to the test customer.
 2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
@@ -5616,7 +5610,7 @@
       </c>
       <c r="H66" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; at least 3 templates exist that are NOT yet linked to the test customer.
+          <t>1. At least 3 templates exist that are NOT yet linked to the test customer.
 2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
@@ -5688,7 +5682,7 @@
       </c>
       <c r="H67" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the location has: (a) a template already linked to this customer, (b) an unlinked Fee/Discount template, and (c) an unlinked Processing Fee template.
+          <t>1. The location has: (a) a template already linked to this customer, (b) an unlinked Fee/Discount template, and (c) an unlinked Processing Fee template.
 2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
@@ -5759,7 +5753,7 @@
       </c>
       <c r="H68" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; every location template is already linked to the test customer (or the location has no templates).</t>
+          <t>1. Every location template is already linked to the test customer (or the location has no templates).</t>
         </is>
       </c>
       <c r="I68" s="15" t="inlineStr">
@@ -5823,7 +5817,7 @@
       </c>
       <c r="H69" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the customer has at least 1 default fee/discount.</t>
+          <t>1. The customer has at least 1 default fee/discount.</t>
         </is>
       </c>
       <c r="I69" s="18" t="inlineStr">
@@ -5895,7 +5889,7 @@
       </c>
       <c r="H70" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; the customer has zero default fees/discounts.</t>
+          <t>1. The customer has zero default fees/discounts.</t>
         </is>
       </c>
       <c r="I70" s="15" t="inlineStr">
@@ -5960,7 +5954,7 @@
       </c>
       <c r="H71" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the customer has a default "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%, non-taxable).</t>
+          <t>1. The customer has a default "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%, non-taxable).</t>
         </is>
       </c>
       <c r="I71" s="18" t="inlineStr">
@@ -6031,7 +6025,7 @@
       </c>
       <c r="H72" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; the customer has a default "ZZAUTOTEST 10% Fee" (Fee, % of Subtotal, 10%, taxable).</t>
+          <t>1. The customer has a default "ZZAUTOTEST 10% Fee" (Fee, % of Subtotal, 10%, taxable).</t>
         </is>
       </c>
       <c r="I72" s="15" t="inlineStr">
@@ -6101,7 +6095,7 @@
       </c>
       <c r="H73" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the customer has a default "ZZAUTOTEST Fleet Discount".
+          <t>1. The customer has a default "ZZAUTOTEST Fleet Discount".
 2. An OPEN work order for that customer already carries the auto-added adjustment from this default.</t>
         </is>
       </c>
@@ -6168,7 +6162,7 @@
       </c>
       <c r="H74" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a template "ZZAUTOTEST Fleet Discount" is a default on the customer AND has been auto-added to an existing OPEN work order.</t>
+          <t>1. A template "ZZAUTOTEST Fleet Discount" is a default on the customer AND has been auto-added to an existing OPEN work order.</t>
         </is>
       </c>
       <c r="I74" s="15" t="inlineStr">
@@ -6239,7 +6233,7 @@
       </c>
       <c r="H75" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a disposable ZZAUTOTEST customer has at least 1 default fee/discount linked.</t>
+          <t>1. A disposable ZZAUTOTEST customer has at least 1 default fee/discount linked.</t>
         </is>
       </c>
       <c r="I75" s="18" t="inlineStr">
@@ -6304,7 +6298,7 @@
       </c>
       <c r="H76" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; the location has exactly 2 templates marked auto-apply and 1 template not auto-apply.</t>
+          <t>1. The location has exactly 2 templates marked auto-apply and 1 template not auto-apply.</t>
         </is>
       </c>
       <c r="I76" s="15" t="inlineStr">
@@ -6369,8 +6363,7 @@
       </c>
       <c r="H77" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON.
-2. A ZZAUTOTEST role is assigned to Tech (exact-user-match) with Customer Management: Create &amp; Edit ON but Manage Accounts Payable and Receivable OFF.</t>
+          <t>1. A ZZAUTOTEST role is assigned to Tech (exact-user-match) with Customer Management: Create &amp; Edit ON but Manage Accounts Payable and Receivable OFF.</t>
         </is>
       </c>
       <c r="I77" s="18" t="inlineStr">
@@ -6440,7 +6433,7 @@
       </c>
       <c r="H78" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a template "ZZAUTOTEST Env Fee" is marked auto-apply at the location AND is a default on the test customer.</t>
+          <t>1. A template "ZZAUTOTEST Env Fee" is marked auto-apply at the location AND is a default on the test customer.</t>
         </is>
       </c>
       <c r="I78" s="15" t="inlineStr">
@@ -6509,7 +6502,7 @@
       </c>
       <c r="H79" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a way to force a server error (e.g., simulate a network/API failure) on the add or remove call.</t>
+          <t>1. A way to force a server error (e.g., simulate a network/API failure) on the add or remove call.</t>
         </is>
       </c>
       <c r="I79" s="18" t="inlineStr">
@@ -6578,7 +6571,7 @@
       </c>
       <c r="H80" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; you have Settings → Finance access.</t>
+          <t>1. You have Settings → Finance access.</t>
         </is>
       </c>
       <c r="I80" s="15" t="inlineStr">
@@ -6647,7 +6640,7 @@
       </c>
       <c r="H81" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the location has at least 1 template.</t>
+          <t>1. The location has at least 1 template.</t>
         </is>
       </c>
       <c r="I81" s="18" t="inlineStr">
@@ -6713,7 +6706,7 @@
       </c>
       <c r="H82" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; you are on Administration → Service → Fees &amp; Discounts.</t>
+          <t>1. You are on Administration → Service → Fees &amp; Discounts.</t>
         </is>
       </c>
       <c r="I82" s="15" t="inlineStr">
@@ -6786,7 +6779,7 @@
       </c>
       <c r="H83" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts page.</t>
+          <t>1. On the admin Fees &amp; Discounts page.</t>
         </is>
       </c>
       <c r="I83" s="18" t="inlineStr">
@@ -6852,7 +6845,7 @@
       </c>
       <c r="H84" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; you can create a template and then a new work order at the same location.</t>
+          <t>1. You can create a template and then a new work order at the same location.</t>
         </is>
       </c>
       <c r="I84" s="15" t="inlineStr">
@@ -6919,7 +6912,7 @@
       </c>
       <c r="H85" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Fee template "ZZAUTOTEST Shop Fee" exists.</t>
+          <t>1. A Fee template "ZZAUTOTEST Shop Fee" exists.</t>
         </is>
       </c>
       <c r="I85" s="18" t="inlineStr">
@@ -6986,7 +6979,7 @@
       </c>
       <c r="H86" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a template that is NOT a default for any customer exists.</t>
+          <t>1. A template that is NOT a default for any customer exists.</t>
         </is>
       </c>
       <c r="I86" s="15" t="inlineStr">
@@ -7056,7 +7049,7 @@
       </c>
       <c r="H87" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a template is set as a default for exactly 2 customers.</t>
+          <t>1. A template is set as a default for exactly 2 customers.</t>
         </is>
       </c>
       <c r="I87" s="18" t="inlineStr">
@@ -7120,7 +7113,7 @@
       </c>
       <c r="H88" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a template has been applied to an OPEN work order as an adjustment.</t>
+          <t>1. A template has been applied to an OPEN work order as an adjustment.</t>
         </is>
       </c>
       <c r="I88" s="15" t="inlineStr">
@@ -7185,7 +7178,7 @@
       </c>
       <c r="H89" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the location has: a "% of Labor Total" template, a "% of Parts Total" template, and a Flat Amount template.
+          <t>1. The location has: a "% of Labor Total" template, a "% of Parts Total" template, and a Flat Amount template.
 2. A work order with at least one labor line and one part exists.</t>
         </is>
       </c>
@@ -7259,7 +7252,7 @@
       </c>
       <c r="H90" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts create dialog.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="I90" s="15" t="inlineStr">
@@ -7330,7 +7323,7 @@
       </c>
       <c r="H91" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; the location has zero templates.</t>
+          <t>1. The location has zero templates.</t>
         </is>
       </c>
       <c r="I91" s="18" t="inlineStr">
@@ -7394,7 +7387,7 @@
       </c>
       <c r="H92" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts create dialog.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="I92" s="15" t="inlineStr">
@@ -7459,7 +7452,7 @@
       </c>
       <c r="H93" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts create dialog with Type = Fee or Discount.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog with Type = Fee or Discount.</t>
         </is>
       </c>
       <c r="I93" s="18" t="inlineStr">
@@ -7528,7 +7521,7 @@
       </c>
       <c r="H94" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a way to force a save failure on the template create/edit call.</t>
+          <t>1. A way to force a save failure on the template create/edit call.</t>
         </is>
       </c>
       <c r="I94" s="15" t="inlineStr">
@@ -7592,8 +7585,7 @@
       </c>
       <c r="H95" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON.
-2. A ZZAUTOTEST role is assigned to Tech (exact-user-match) WITHOUT Settings → Finance.</t>
+          <t>1. A ZZAUTOTEST role is assigned to Tech (exact-user-match) WITHOUT Settings → Finance.</t>
         </is>
       </c>
       <c r="I95" s="18" t="inlineStr">
@@ -7661,7 +7653,7 @@
       </c>
       <c r="H96" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts create dialog.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="I96" s="15" t="inlineStr">
@@ -7726,7 +7718,7 @@
       </c>
       <c r="H97" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts create dialog.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="I97" s="18" t="inlineStr">
@@ -7794,7 +7786,7 @@
       </c>
       <c r="H98" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin Fees &amp; Discounts create dialog with Type = "Processing Fee".</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog with Type = "Processing Fee".</t>
         </is>
       </c>
       <c r="I98" s="15" t="inlineStr">
@@ -7860,7 +7852,7 @@
       </c>
       <c r="H99" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin create dialog with Type = Processing Fee.</t>
+          <t>1. On the admin create dialog with Type = Processing Fee.</t>
         </is>
       </c>
       <c r="I99" s="18" t="inlineStr">
@@ -7924,7 +7916,7 @@
       </c>
       <c r="H100" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; on the admin create dialog with Type = Processing Fee.</t>
+          <t>1. On the admin create dialog with Type = Processing Fee.</t>
         </is>
       </c>
       <c r="I100" s="15" t="inlineStr">
@@ -7995,7 +7987,7 @@
       </c>
       <c r="H101" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Processing Fee template exists.
+          <t>1. A Processing Fee template exists.
 2. An open work order is available.</t>
         </is>
       </c>
@@ -8065,7 +8057,7 @@
       </c>
       <c r="H102" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Processing Fee template "ZZAUTOTEST Proc Fee" (Flat Amount $5.00, taxable Yes) is marked auto-apply.</t>
+          <t>1. A Processing Fee template "ZZAUTOTEST Proc Fee" (Flat Amount $5.00, taxable Yes) is marked auto-apply.</t>
         </is>
       </c>
       <c r="I102" s="15" t="inlineStr">
@@ -8130,7 +8122,7 @@
       </c>
       <c r="H103" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Processing Fee template is set as a default on the test customer.</t>
+          <t>1. A Processing Fee template is set as a default on the test customer.</t>
         </is>
       </c>
       <c r="I103" s="18" t="inlineStr">
@@ -8195,7 +8187,7 @@
       </c>
       <c r="H104" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; an open WO carries a Processing Fee (via auto-apply or customer default).</t>
+          <t>1. An open WO carries a Processing Fee (via auto-apply or customer default).</t>
         </is>
       </c>
       <c r="I104" s="15" t="inlineStr">
@@ -8265,7 +8257,7 @@
       </c>
       <c r="H105" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Processing Fee template "ZZAUTOTEST 3% Proc" (% of Grand Total, 3%, taxable Yes) auto-applies.
+          <t>1. A Processing Fee template "ZZAUTOTEST 3% Proc" (% of Grand Total, 3%, taxable Yes) auto-applies.
 2. A work order exists whose net subtotal (after line-level adjustments) = $300.00 and pre-fee tax = $24.00 (so Grand Total base = $324.00).</t>
         </is>
       </c>
@@ -8336,7 +8328,7 @@
       </c>
       <c r="H106" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; ability to submit template data (via UI edge case or API) for a Processing Fee carrying a Max Amount, or a method other than Flat Amount / % of Grand Total.</t>
+          <t>1. Ability to submit template data (via UI edge case or API) for a Processing Fee carrying a Max Amount, or a method other than Flat Amount / % of Grand Total.</t>
         </is>
       </c>
       <c r="I106" s="15" t="inlineStr">
@@ -8405,7 +8397,7 @@
       </c>
       <c r="H107" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Processing Fee template exists and is on a WO.</t>
+          <t>1. A Processing Fee template exists and is on a WO.</t>
         </is>
       </c>
       <c r="I107" s="18" t="inlineStr">
@@ -8470,7 +8462,7 @@
       </c>
       <c r="H108" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a Processing Fee template auto-applied to an existing OPEN work order (e.g. Flat $5.00).</t>
+          <t>1. A Processing Fee template auto-applied to an existing OPEN work order (e.g. Flat $5.00).</t>
         </is>
       </c>
       <c r="I108" s="15" t="inlineStr">
@@ -8535,7 +8527,7 @@
       </c>
       <c r="H109" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; two Processing Fee templates (both % of Grand Total) auto-apply to one work order.
+          <t>1. Two Processing Fee templates (both % of Grand Total) auto-apply to one work order.
 2. Net subtotal $300.00, pre-fee tax $24.00 → Grand Total base $324.00.</t>
         </is>
       </c>
@@ -8601,7 +8593,7 @@
       </c>
       <c r="H110" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; ability to submit a Processing Fee with a non-empty minimum amount (no UI control exists; guard for external data).</t>
+          <t>1. Ability to submit a Processing Fee with a non-empty minimum amount (no UI control exists; guard for external data).</t>
         </is>
       </c>
       <c r="I110" s="15" t="inlineStr">
@@ -8668,7 +8660,7 @@
       </c>
       <c r="H111" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a work order has whole-WO and line-level adjustments and can produce both an estimate and an invoice.</t>
+          <t>1. A work order has whole-WO and line-level adjustments and can produce both an estimate and an invoice.</t>
         </is>
       </c>
       <c r="I111" s="18" t="inlineStr">
@@ -8737,7 +8729,7 @@
       </c>
       <c r="H112" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has a labor line with a "Shop Supply Fee" (% of Labor Total, fee) and a labor-line discount.</t>
+          <t>1. A WO has a labor line with a "Shop Supply Fee" (% of Labor Total, fee) and a labor-line discount.</t>
         </is>
       </c>
       <c r="I112" s="15" t="inlineStr">
@@ -8803,7 +8795,7 @@
       </c>
       <c r="H113" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO part has a percentage part-line adjustment and another part has a Flat Amount part-line adjustment.</t>
+          <t>1. A WO part has a percentage part-line adjustment and another part has a Flat Amount part-line adjustment.</t>
         </is>
       </c>
       <c r="I113" s="18" t="inlineStr">
@@ -8868,7 +8860,7 @@
       </c>
       <c r="H114" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has both a fee and a discount adjustment.</t>
+          <t>1. A WO has both a fee and a discount adjustment.</t>
         </is>
       </c>
       <c r="I114" s="15" t="inlineStr">
@@ -8938,7 +8930,7 @@
       </c>
       <c r="H115" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has 3 whole-WO adjustments created in a known order, including a % of Subtotal and a Flat Amount.</t>
+          <t>1. A WO has 3 whole-WO adjustments created in a known order, including a % of Subtotal and a Flat Amount.</t>
         </is>
       </c>
       <c r="I115" s="18" t="inlineStr">
@@ -9004,7 +8996,7 @@
       </c>
       <c r="H116" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has three separate "Shop Supply Fee" line-level fees (same name+type) across different lines.</t>
+          <t>1. A WO has three separate "Shop Supply Fee" line-level fees (same name+type) across different lines.</t>
         </is>
       </c>
       <c r="I116" s="15" t="inlineStr">
@@ -9073,7 +9065,7 @@
       </c>
       <c r="H117" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO carries a % of Grand Total Processing Fee.</t>
+          <t>1. A WO carries a % of Grand Total Processing Fee.</t>
         </is>
       </c>
       <c r="I117" s="18" t="inlineStr">
@@ -9136,7 +9128,7 @@
       </c>
       <c r="H118" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO whose total shop supplies = $0.00.</t>
+          <t>1. A WO whose total shop supplies = $0.00.</t>
         </is>
       </c>
       <c r="I118" s="15" t="inlineStr">
@@ -9202,7 +9194,7 @@
       </c>
       <c r="H119" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO that currently has $0.00 shop supplies (Shop Supplies hidden on customer views).</t>
+          <t>1. A WO that currently has $0.00 shop supplies (Shop Supplies hidden on customer views).</t>
         </is>
       </c>
       <c r="I119" s="18" t="inlineStr">
@@ -9266,7 +9258,7 @@
       </c>
       <c r="H120" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO labor line with an adjustment is set to declined/not-billable.</t>
+          <t>1. A WO labor line with an adjustment is set to declined/not-billable.</t>
         </is>
       </c>
       <c r="I120" s="15" t="inlineStr">
@@ -9331,7 +9323,7 @@
       </c>
       <c r="H121" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO with labor, parts, shop supplies (&gt; $0.00), and whole-WO adjustments.</t>
+          <t>1. A WO with labor, parts, shop supplies (&gt; $0.00), and whole-WO adjustments.</t>
         </is>
       </c>
       <c r="I121" s="18" t="inlineStr">
@@ -9394,7 +9386,7 @@
       </c>
       <c r="H122" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; location has an active QuickBooks connection with mapped Fee and Discount items.
+          <t>1. Location has an active QuickBooks connection with mapped Fee and Discount items.
 2. A WO with one fee (+$10.00) and one discount (−$20.00) is invoiced.</t>
         </is>
       </c>
@@ -9465,7 +9457,7 @@
       </c>
       <c r="H123" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected with a mapped Fee item and Discount item.
+          <t>1. QuickBooks connected with a mapped Fee item and Discount item.
 2. A WO has a fee named "Hazmat Disposal Fee"; the WO is invoiced.</t>
         </is>
       </c>
@@ -9531,7 +9523,7 @@
       </c>
       <c r="H124" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; a WO has an adjustment that resolves to $0.00 (e.g. target not billable, or $0 base).</t>
+          <t>1. QuickBooks connected; a WO has an adjustment that resolves to $0.00 (e.g. target not billable, or $0 base).</t>
         </is>
       </c>
       <c r="I124" s="15" t="inlineStr">
@@ -9596,7 +9588,7 @@
       </c>
       <c r="H125" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; the Fee item is NOT mapped in Settings → QuickBooks.
+          <t>1. QuickBooks connected; the Fee item is NOT mapped in Settings → QuickBooks.
 2. The Discount item IS mapped.
 3. An open WO is available.</t>
         </is>
@@ -9663,7 +9655,7 @@
       </c>
       <c r="H126" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; the Discount item is NOT mapped; the Fee item IS mapped.
+          <t>1. QuickBooks connected; the Discount item is NOT mapped; the Fee item IS mapped.
 2. An open WO is available.</t>
         </is>
       </c>
@@ -9729,7 +9721,7 @@
       </c>
       <c r="H127" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; Fee item UNMAPPED.</t>
+          <t>1. QuickBooks connected; Fee item UNMAPPED.</t>
         </is>
       </c>
       <c r="I127" s="18" t="inlineStr">
@@ -9796,7 +9788,7 @@
       </c>
       <c r="H128" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; Fee item UNMAPPED.</t>
+          <t>1. QuickBooks connected; Fee item UNMAPPED.</t>
         </is>
       </c>
       <c r="I128" s="15" t="inlineStr">
@@ -9861,7 +9853,7 @@
       </c>
       <c r="H129" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; scenario A: QuickBooks connected with Fee item unmapped; scenario B: QuickBooks NOT connected.</t>
+          <t>1. Scenario A: QuickBooks connected with Fee item unmapped; scenario B: QuickBooks NOT connected.</t>
         </is>
       </c>
       <c r="I129" s="18" t="inlineStr">
@@ -9926,7 +9918,7 @@
       </c>
       <c r="H130" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected with mapped Fee item; a WO with a fee is ready to invoice/sync.</t>
+          <t>1. QuickBooks connected with mapped Fee item; a WO with a fee is ready to invoice/sync.</t>
         </is>
       </c>
       <c r="I130" s="15" t="inlineStr">
@@ -9993,7 +9985,7 @@
       </c>
       <c r="H131" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected with a location Class set; a WO with fees/discounts is invoiced.</t>
+          <t>1. QuickBooks connected with a location Class set; a WO with fees/discounts is invoiced.</t>
         </is>
       </c>
       <c r="I131" s="18" t="inlineStr">
@@ -10061,7 +10053,7 @@
       </c>
       <c r="H132" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; the location's Class has been deleted/deactivated in QuickBooks.</t>
+          <t>1. QuickBooks connected; the location's Class has been deleted/deactivated in QuickBooks.</t>
         </is>
       </c>
       <c r="I132" s="15" t="inlineStr">
@@ -10125,7 +10117,7 @@
       </c>
       <c r="H133" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; a WO has $100.00 taxable parts and $10.00 tax.</t>
+          <t>1. QuickBooks connected; a WO has $100.00 taxable parts and $10.00 tax.</t>
         </is>
       </c>
       <c r="I133" s="18" t="inlineStr">
@@ -10195,7 +10187,7 @@
       </c>
       <c r="H134" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; a WO where stacked MULTIPLE discount lines drive the net subtotal below $0.00 (floor applies).</t>
+          <t>1. QuickBooks connected; a WO where stacked MULTIPLE discount lines drive the net subtotal below $0.00 (floor applies).</t>
         </is>
       </c>
       <c r="I134" s="15" t="inlineStr">
@@ -10261,7 +10253,7 @@
       </c>
       <c r="H135" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO where discounts will exceed the net subtotal.</t>
+          <t>1. A WO where discounts will exceed the net subtotal.</t>
         </is>
       </c>
       <c r="I135" s="18" t="inlineStr">
@@ -10326,7 +10318,7 @@
       </c>
       <c r="H136" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; a WO where the floor applied (from FD-QB-012, $50.00 excess).</t>
+          <t>1. QuickBooks connected; a WO where the floor applied (from FD-QB-012, $50.00 excess).</t>
         </is>
       </c>
       <c r="I136" s="15" t="inlineStr">
@@ -10392,7 +10384,7 @@
       </c>
       <c r="H137" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; QuickBooks connected; a WO has one taxable fee and one non-taxable fee; the WO is invoiced.</t>
+          <t>1. QuickBooks connected; a WO has one taxable fee and one non-taxable fee; the WO is invoiced.</t>
         </is>
       </c>
       <c r="I137" s="18" t="inlineStr">
@@ -10456,7 +10448,7 @@
       </c>
       <c r="H138" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; you have View History Logs and can add/edit/remove adjustments on an open WO.</t>
+          <t>1. You have View History Logs and can add/edit/remove adjustments on an open WO.</t>
         </is>
       </c>
       <c r="I138" s="15" t="inlineStr">
@@ -10523,7 +10515,7 @@
       </c>
       <c r="H139" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has (a) a whole-WO 10% fee named "Env Fee", (b) a labor-line $5.00 flat fee, (c) a part-line discount.</t>
+          <t>1. A WO has (a) a whole-WO 10% fee named "Env Fee", (b) a labor-line $5.00 flat fee, (c) a part-line discount.</t>
         </is>
       </c>
       <c r="I139" s="18" t="inlineStr">
@@ -10594,7 +10586,7 @@
       </c>
       <c r="H140" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has at least one whole-WO adjustment and one line-level adjustment logged.</t>
+          <t>1. A WO has at least one whole-WO adjustment and one line-level adjustment logged.</t>
         </is>
       </c>
       <c r="I140" s="15" t="inlineStr">
@@ -10658,7 +10650,7 @@
       </c>
       <c r="H141" s="18" t="inlineStr">
         <is>
-          <t>1. A WO already has fee/discount history entries recorded while the flag was ON.
+          <t>1. A WO already has fee/discount history entries.
 2. The Fees &amp; Discounts feature flag is then turned OFF for the org.</t>
         </is>
       </c>
@@ -10728,7 +10720,7 @@
       </c>
       <c r="H142" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has fee/discount history entries.
+          <t>1. A WO has fee/discount history entries.
 2. A ZZAUTOTEST role is assigned to Tech with View History Logs ON but See Financial Data OFF (exact-user-match).</t>
         </is>
       </c>
@@ -10799,7 +10791,7 @@
       </c>
       <c r="H143" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has fee/discount history.
+          <t>1. A WO has fee/discount history.
 2. A ZZAUTOTEST role is assigned to Tech WITHOUT View History Logs (exact-user-match).</t>
         </is>
       </c>
@@ -10868,7 +10860,7 @@
       </c>
       <c r="H144" s="15" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO carries a Processing Fee (via auto-apply or customer default).</t>
+          <t>1. A WO carries a Processing Fee (via auto-apply or customer default).</t>
         </is>
       </c>
       <c r="I144" s="15" t="inlineStr">
@@ -10938,7 +10930,7 @@
       </c>
       <c r="H145" s="18" t="inlineStr">
         <is>
-          <t>1. Flag ON; a WO has a whole-WO 10% fee.</t>
+          <t>1. A WO has a whole-WO 10% fee.</t>
         </is>
       </c>
       <c r="I145" s="18" t="inlineStr">
@@ -11002,9 +10994,8 @@
       </c>
       <c r="H146" s="15" t="inlineStr">
         <is>
-          <t>1. Fees &amp; Discounts feature flag is ON for the organization.
-2. You are signed in with a role that has See Financial Data and Work Orders: Create and Edit.
-3. An open work order (not Invoiced/Paid, not in history mode) exists whose relevant base equals exactly $150.00 (e.g. net labor total = $150.00). Mark any throwaway data ZZAUTOTEST.</t>
+          <t>1. You are signed in with a role that has See Financial Data and Work Orders: Create and Edit.
+2. An open work order (not Invoiced/Paid, not in history mode) exists whose relevant base equals exactly $150.00 (e.g. net labor total = $150.00). Mark any throwaway data ZZAUTOTEST.</t>
         </is>
       </c>
       <c r="I146" s="15" t="inlineStr">
@@ -11078,9 +11069,8 @@
       </c>
       <c r="H147" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and Work Orders: Create and Edit.
-3. An open work order whose target base equals exactly $33.33.</t>
+          <t>1. Role has See Financial Data and Work Orders: Create and Edit.
+2. An open work order whose target base equals exactly $33.33.</t>
         </is>
       </c>
       <c r="I147" s="18" t="inlineStr">
@@ -11154,9 +11144,8 @@
       </c>
       <c r="H148" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data plus the matching change permission.
-3. An open work order with at least one labor line.</t>
+          <t>1. Role has See Financial Data plus the matching change permission.
+2. An open work order with at least one labor line.</t>
         </is>
       </c>
       <c r="I148" s="15" t="inlineStr">
@@ -11227,9 +11216,8 @@
       </c>
       <c r="H149" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and Work Order Lines: Create and Edit.
-3. An open work order with a part whose quantity = 3.</t>
+          <t>1. Role has See Financial Data and Work Order Lines: Create and Edit.
+2. An open work order with a part whose quantity = 3.</t>
         </is>
       </c>
       <c r="I149" s="18" t="inlineStr">
@@ -11301,9 +11289,8 @@
       </c>
       <c r="H150" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order.</t>
         </is>
       </c>
       <c r="I150" s="15" t="inlineStr">
@@ -11376,9 +11363,8 @@
       </c>
       <c r="H151" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order.</t>
         </is>
       </c>
       <c r="I151" s="18" t="inlineStr">
@@ -11449,9 +11435,8 @@
       </c>
       <c r="H152" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order whose target base = $100.00.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order whose target base = $100.00.</t>
         </is>
       </c>
       <c r="I152" s="15" t="inlineStr">
@@ -11524,10 +11509,9 @@
       </c>
       <c r="H153" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order whose target base = $100.00.
-4. Note: a $0 Max Amount can normally only come from old data — an entered 0 is treated as empty in the current dialogs (S2-R25).</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order whose target base = $100.00.
+3. Note: a $0 Max Amount can normally only come from old data — an entered 0 is treated as empty in the current dialogs (S2-R25).</t>
         </is>
       </c>
       <c r="I153" s="18" t="inlineStr">
@@ -11598,9 +11582,8 @@
       </c>
       <c r="H154" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order with a target line whose base is $0.00 (e.g. a declined/not-billable labor line, §5-R12).</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order with a target line whose base is $0.00 (e.g. a declined/not-billable labor line, §5-R12).</t>
         </is>
       </c>
       <c r="I154" s="15" t="inlineStr">
@@ -11671,9 +11654,8 @@
       </c>
       <c r="H155" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order where an earlier discount has already driven a net total to or below $0 for a whole-WO percentage base.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order where an earlier discount has already driven a net total to or below $0 for a whole-WO percentage base.</t>
         </is>
       </c>
       <c r="I155" s="18" t="inlineStr">
@@ -11743,9 +11725,8 @@
       </c>
       <c r="H156" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order for a taxable customer with a known tax rate and a taxable base.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order for a taxable customer with a known tax rate and a taxable base.</t>
         </is>
       </c>
       <c r="I156" s="15" t="inlineStr">
@@ -11817,9 +11798,8 @@
       </c>
       <c r="H157" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data plus both change permissions.
-3. An open work order with gross labor = $200.00 and gross parts = $100.00 (spec worked example).</t>
+          <t>1. Role has See Financial Data plus both change permissions.
+2. An open work order with gross labor = $200.00 and gross parts = $100.00 (spec worked example).</t>
         </is>
       </c>
       <c r="I157" s="18" t="inlineStr">
@@ -11891,10 +11871,9 @@
       </c>
       <c r="H158" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has Settings → Finance to create the template and See Financial Data to view amounts.
-3. A Processing Fee template exists: Type = Processing Fee, Calculation type = % of Grand Total, Percent = 3%, marked auto-apply or set as a customer default (a Processing Fee cannot be added to a WO by hand, S8-R16).
-4. An open work order whose net subtotal after line discounts = $300.00 with pre-fee tax = $24.00 (Grand Total base = $324.00).</t>
+          <t>1. Role has Settings → Finance to create the template and See Financial Data to view amounts.
+2. A Processing Fee template exists: Type = Processing Fee, Calculation type = % of Grand Total, Percent = 3%, marked auto-apply or set as a customer default (a Processing Fee cannot be added to a WO by hand, S8-R16).
+3. An open work order whose net subtotal after line discounts = $300.00 with pre-fee tax = $24.00 (Grand Total base = $324.00).</t>
         </is>
       </c>
       <c r="I158" s="15" t="inlineStr">
@@ -11965,9 +11944,8 @@
       </c>
       <c r="H159" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has Settings → Finance and See Financial Data.
-3. On the template admin page, open the Processing Fee template create/edit dialog.</t>
+          <t>1. Role has Settings → Finance and See Financial Data.
+2. On the template admin page, open the Processing Fee template create/edit dialog.</t>
         </is>
       </c>
       <c r="I159" s="18" t="inlineStr">
@@ -12040,10 +12018,9 @@
       </c>
       <c r="H160" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order with $100.00 taxable parts and $10.00 tax (spec worked example).
-4. Location has an active QuickBooks connection (to verify the credit memo).</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order with $100.00 taxable parts and $10.00 tax (spec worked example).
+3. Location has an active QuickBooks connection (to verify the credit memo).</t>
         </is>
       </c>
       <c r="I160" s="15" t="inlineStr">
@@ -12117,9 +12094,8 @@
       </c>
       <c r="H161" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order with $100.00 taxable parts and $10.00 tax (same base as FD-CALC-015).</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order with $100.00 taxable parts and $10.00 tax (same base as FD-CALC-015).</t>
         </is>
       </c>
       <c r="I161" s="18" t="inlineStr">
@@ -12191,10 +12167,9 @@
       </c>
       <c r="H162" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. Location has an active QuickBooks connection.
-4. An open work order with a small net subtotal and two or more discount lines whose combined size exceeds it.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. Location has an active QuickBooks connection.
+3. An open work order with a small net subtotal and two or more discount lines whose combined size exceeds it.</t>
         </is>
       </c>
       <c r="I162" s="15" t="inlineStr">
@@ -12266,9 +12241,8 @@
       </c>
       <c r="H163" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. A work order (and a part sale, and a customer) already has adjustments to view.
-3. Two ZZAUTOTEST custom roles ready: Role A WITH See Financial Data; Role B WITHOUT See Financial Data (otherwise identical). Use exact-user-match when assigning to Tech (Tech /change staff_id 6fb22c1b-…).</t>
+          <t>1. A work order (and a part sale, and a customer) already has adjustments to view.
+2. Two ZZAUTOTEST custom roles ready: Role A WITH See Financial Data; Role B WITHOUT See Financial Data (otherwise identical). Use exact-user-match when assigning to Tech (Tech /change staff_id 6fb22c1b-…).</t>
         </is>
       </c>
       <c r="I163" s="18" t="inlineStr">
@@ -12340,9 +12314,8 @@
       </c>
       <c r="H164" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. An open work order.
-3. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Orders: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
+          <t>1. An open work order.
+2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Orders: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I164" s="15" t="inlineStr">
@@ -12413,9 +12386,8 @@
       </c>
       <c r="H165" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. An open work order with a labor line and a part.
-3. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Order Lines: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
+          <t>1. An open work order with a labor line and a part.
+2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Order Lines: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I165" s="18" t="inlineStr">
@@ -12486,9 +12458,8 @@
       </c>
       <c r="H166" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. An open part sale with at least one part.
-3. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Part Sales: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
+          <t>1. An open part sale with at least one part.
+2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Part Sales: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I166" s="15" t="inlineStr">
@@ -12559,9 +12530,8 @@
       </c>
       <c r="H167" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. An open work order.
-3. A ZZAUTOTEST role that HAS Work Orders: Create and Edit (and/or Work Order Lines / Part Sales Create and Edit) but has See Financial Data OFF. Assign by exact-user-match to Tech.</t>
+          <t>1. An open work order.
+2. A ZZAUTOTEST role that HAS Work Orders: Create and Edit (and/or Work Order Lines / Part Sales Create and Edit) but has See Financial Data OFF. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I167" s="18" t="inlineStr">
@@ -12632,9 +12602,8 @@
       </c>
       <c r="H168" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. An open work order with an existing whole-WO adjustment.
-3. A ZZAUTOTEST role with See Financial Data ON and Work Orders: Create and Edit ON, but with the Work Orders "Delete" permission OFF. Assign by exact-user-match to Tech.</t>
+          <t>1. An open work order with an existing whole-WO adjustment.
+2. A ZZAUTOTEST role with See Financial Data ON and Work Orders: Create and Edit ON, but with the Work Orders "Delete" permission OFF. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I168" s="15" t="inlineStr">
@@ -12705,8 +12674,7 @@
       </c>
       <c r="H169" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Two ZZAUTOTEST roles: Role A WITH Settings → Finance; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
+          <t>1. Two ZZAUTOTEST roles: Role A WITH Settings → Finance; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I169" s="18" t="inlineStr">
@@ -12777,9 +12745,8 @@
       </c>
       <c r="H170" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. A customer exists.
-3. Three ZZAUTOTEST roles: (A) both permissions ON; (B) Customer Management ON but Manage AP/AR OFF; (C) Manage AP/AR ON but Customer Management OFF. Assign by exact-user-match to Tech.</t>
+          <t>1. A customer exists.
+2. Three ZZAUTOTEST roles: (A) both permissions ON; (B) Customer Management ON but Manage AP/AR OFF; (C) Manage AP/AR ON but Customer Management OFF. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="I170" s="15" t="inlineStr">
@@ -13001,9 +12968,8 @@
       </c>
       <c r="H173" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. The user has all F&amp;D permissions (so only the WO state should block).
-3. An Invoiced or Paid work order, and separately a way to enter history mode.</t>
+          <t>1. The user has all F&amp;D permissions (so only the WO state should block).
+2. An Invoiced or Paid work order, and separately a way to enter history mode.</t>
         </is>
       </c>
       <c r="I173" s="18" t="inlineStr">
@@ -13148,7 +13114,7 @@
       </c>
       <c r="H175" s="18" t="inlineStr">
         <is>
-          <t>1. A work order already has fee/discount history entries created while the flag was ON.
+          <t>1. A work order already has fee/discount history entries.
 2. The user has View History Logs.
 3. Ability to set the FeesAndDiscounts flag OFF.</t>
         </is>
@@ -13220,9 +13186,8 @@
       </c>
       <c r="H176" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON for the org.
-2. Two ZZAUTOTEST roles: one with the F&amp;D-relevant permissions, one without.
-3. An open work order.</t>
+          <t>1. Two ZZAUTOTEST roles: one with the F&amp;D-relevant permissions, one without.
+2. An open work order.</t>
         </is>
       </c>
       <c r="I176" s="15" t="inlineStr">
@@ -13293,9 +13258,8 @@
       </c>
       <c r="H177" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. An open work order; open the Add Fee / Discount dialog.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. An open work order; open the Add Fee / Discount dialog.</t>
         </is>
       </c>
       <c r="I177" s="18" t="inlineStr">
@@ -13368,9 +13332,8 @@
       </c>
       <c r="H178" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. Add dialog open with Name and Type and Calculation type filled.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. Add dialog open with Name and Type and Calculation type filled.</t>
         </is>
       </c>
       <c r="I178" s="15" t="inlineStr">
@@ -13441,9 +13404,8 @@
       </c>
       <c r="H179" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. Add dialog open with Type, Calculation type, and a valid Amount filled.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. Add dialog open with Type, Calculation type, and a valid Amount filled.</t>
         </is>
       </c>
       <c r="I179" s="18" t="inlineStr">
@@ -13514,9 +13476,8 @@
       </c>
       <c r="H180" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. Add dialog open.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. Add dialog open.</t>
         </is>
       </c>
       <c r="I180" s="15" t="inlineStr">
@@ -13588,9 +13549,8 @@
       </c>
       <c r="H181" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. Add dialog open with Name, Type, Calculation type set.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. Add dialog open with Name, Type, Calculation type set.</t>
         </is>
       </c>
       <c r="I181" s="18" t="inlineStr">
@@ -13659,9 +13619,8 @@
       </c>
       <c r="H182" s="15" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. Role has See Financial Data and the matching change permission.
-3. Add dialog open.</t>
+          <t>1. Role has See Financial Data and the matching change permission.
+2. Add dialog open.</t>
         </is>
       </c>
       <c r="I182" s="15" t="inlineStr">
@@ -13732,9 +13691,8 @@
       </c>
       <c r="H183" s="18" t="inlineStr">
         <is>
-          <t>1. Feature flag ON.
-2. A template at the location is marked auto-apply (S7-R5).
-3. The SAME template is also set as a default for a customer (S9-R2).</t>
+          <t>1. A template at the location is marked auto-apply (S7-R5).
+2. The SAME template is also set as a default for a customer (S9-R2).</t>
         </is>
       </c>
       <c r="I183" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Fees & Discounts: apply VIU case-update deviations to TestRail
Applied 10 safe VIU case-update deviations (label/copy/placement drift where
the app behaves acceptably) in-place to live TestRail (update_case, all HTTP
200, re-fetch verified): FD-WO-001, FD-LABOR-001, FD-FIN-004, FD-REMOVE-001,
FD-TMPL-001, FD-TMPL-003, FD-TMPL-004, FD-TMPL-006, FD-TMPL-008, FD-PROC-008.
Updated the matching case JSONs and regenerated the local mirrors
(FeesDiscounts_V1_TestCases.csv/.xlsx + testrail-import CSV/xlsx; 0 VIU,
0 feature-flag, API routing + header unchanged). Held the FDBUG-overlap and
PO-question rows. Audit log: testrail-caseupdate-log.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
+++ b/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
@@ -1019,14 +1019,14 @@
       <c r="I2" s="15" t="inlineStr">
         <is>
           <t>1. Click the ⋯ (More actions) menu at the top-right of the work order toolbar.
-2. Click the menu item 'Add Work Order Fee / Discount'.
+2. Click the menu item 'Add Fee/Discount'.
 3. Observe the dialog title and any subtitle.</t>
         </is>
       </c>
       <c r="J2" s="15" t="inlineStr">
         <is>
-          <t>1. A dialog opens with the title 'New Fee / Discount' (spec S2-R9). In the current design mockup the header reads 'Add new fee/discount' with the WO number (e.g. 'S2-13274') as the context subtitle.
-2. There is NO 'Applying to:' subtitle, because Whole Work Order scope has none (S2-R12).
+          <t>1. A dialog opens with the title 'Add new fee/discount' and the work order number (e.g. 'S2-13274') shown as the context subtitle.
+2. There is NO 'Applying to:' subtitle, because Whole Work Order scope has none.
 3. The scope is Whole Work Order and cannot be changed from inside the dialog (there is no scope dropdown).</t>
         </is>
       </c>
@@ -2112,9 +2112,9 @@
       </c>
       <c r="J17" s="18" t="inlineStr">
         <is>
-          <t>1. The dialog opens locked to Labor Line scope for that specific line (S1-R3).
-2. A grey subtitle reads 'Applying to: Line 1 Labor — Service - Perform LOF and inspection' (S2-R10), or 'Applying to: Line 1 Labor' when the line has no name.
-3. Scope/target cannot be changed inside the dialog (S2-R8).</t>
+          <t>1. The dialog opens locked to Labor Line scope for that specific line.
+2. A grey subtitle reads 'Applying to: {line name}' (e.g. 'Applying to: Service - Perform LOF and inspection'); it does NOT include a 'Line {N} Labor —' prefix.
+3. Scope/target cannot be changed inside the dialog.</t>
         </is>
       </c>
       <c r="K17" s="18" t="inlineStr">
@@ -4105,16 +4105,16 @@
       </c>
       <c r="I45" s="18" t="inlineStr">
         <is>
-          <t>1. Look at the left-sidebar 'Work Order Fee / Discount' card.
+          <t>1. Look at the left-sidebar 'WO Fees &amp; Discounts' card.
 2. Read the listed entries and confirm which scopes appear.
 3. Hover an entry and open its ⋯ menu.</t>
         </is>
       </c>
       <c r="J45" s="18" t="inlineStr">
         <is>
-          <t>1. The card lists ONLY whole-Work-Order adjustments (S3-R3) — line-level adjustments do NOT appear here.
-2. The 'Early Payment Discount' entry shows a signed rate badge '−8%' (S3-R5/R6) and the resolved amount −$857.23 in plain grey, signed (S3-R8).
-3. Hovering shows a ⋯ 3-dot menu with 'Edit' and 'Delete' only (S3-R9), shown only when the WO is open and the user has the change permission.</t>
+          <t>1. The card is titled 'WO Fees &amp; Discounts' and lists ONLY whole-Work-Order adjustments — line-level adjustments do NOT appear here.
+2. The 'Early Payment Discount' entry shows a signed rate badge '−8%' and the resolved amount −$857.23 in plain grey, signed.
+3. Hovering shows a ⋯ 3-dot menu with 'Edit' and 'Remove' only, shown only when the WO is open and the user has the change permission.</t>
         </is>
       </c>
       <c r="K45" s="18" t="inlineStr">
@@ -4961,17 +4961,17 @@
       </c>
       <c r="I57" s="18" t="inlineStr">
         <is>
-          <t>1. On the sidebar 'Work Order Fee / Discount' card, hover the 'Early Payment Discount' entry and open its ⋯ menu.
-2. Click 'Delete'.
+          <t>1. On the sidebar 'WO Fees &amp; Discounts' card, hover the 'Early Payment Discount' entry and open its ⋯ menu.
+2. Click 'Remove'.
 3. Read the confirm dialog.
 4. Click the confirm button.</t>
         </is>
       </c>
       <c r="J57" s="18" t="inlineStr">
         <is>
-          <t>1. A confirm dialog opens titled 'Remove Fee / Discount' with the message 'Remove "Early Payment Discount" from this work order?' and a red 'Remove' confirm button (S3-R11a).
-2. On confirm, the adjustment is removed (S3-R11b).
-3. A success toast reads 'Discount removed' (§7); the entry disappears from the card and the count/totals update.</t>
+          <t>1. A confirm dialog opens titled 'Remove Fee / Discount' with the message 'Are you sure you want to remove this fee?' and a red 'Remove' confirm button.
+2. On confirm, the adjustment is removed.
+3. A success toast confirms removal (observed wording 'Fee removed'; confirm whether it varies to 'Discount removed' by adjustment kind); the entry disappears from the card and the count/totals update.</t>
         </is>
       </c>
       <c r="K57" s="18" t="inlineStr">
@@ -6596,14 +6596,14 @@
       </c>
       <c r="I80" s="15" t="inlineStr">
         <is>
-          <t>1. Go to Administration → Service.
+          <t>1. Go to Administration → Finance.
 2. Locate the Fees &amp; Discounts section.</t>
         </is>
       </c>
       <c r="J80" s="15" t="inlineStr">
         <is>
-          <t>1. A "Fees &amp; Discounts" template page/section is present under Administration → Service.
-2. It appears directly below "Canned Lines".</t>
+          <t>1. A "Fees &amp; Discounts" template page/section is present under Administration → Finance (route /administration/adjustment-templates).
+2. It appears directly below "Payment Methods".</t>
         </is>
       </c>
       <c r="K80" s="15" t="inlineStr">
@@ -6737,16 +6737,16 @@
         <is>
           <t>1. Click "New fee / discount".
 2. Confirm the dialog title reads "New Fee / Discount".
-3. Set Type = "Fee"; Calculation type = "% of Labor Total"; Name = "ZZAUTOTEST Shop Fee"; Percent = 5; leave Max Amount blank; Taxable = "Yes"; leave the auto-apply checkbox unchecked.
+3. Set Type = "Fee"; Calculation type = "% of Labor Total"; Name = "ZZAUTOTEST Shop Fee"; Percent = 5; leave Max Amount blank; leave the Taxable toggle ON; optionally add a Description; leave the "Auto-apply to new work orders" toggle OFF.
 4. Click the confirm button.</t>
         </is>
       </c>
       <c r="J82" s="15" t="inlineStr">
         <is>
-          <t>1. The dialog has fields: Type (Fee/Discount/Processing Fee dropdown), Calculation type, Name (up to 100 chars), Amount or Percent, "Max Amount (Optional)" (percentage methods only), Taxable Yes/No (default Yes), and an "Auto-apply to all new work orders at this location" checkbox.
+          <t>1. The dialog has fields: Type (Fee/Discount/Processing Fee dropdown), Calculation type, Name (up to 100 chars), "$ Default Amount"/Percent, "Max Amount (Optional)" (percentage methods only), a Taxable toggle (default ON), a "Description (Optional)" field (up to 255 chars), and an "Auto-apply to new work orders" toggle.
 2. There is NO scope field (every template is whole-WO).
-3. The confirm button reads exactly "Add Fee / Discount" (fixed label for creation, any type).
-4. On save, a success toast reads exactly "Fee added" and the new template appears in the list.</t>
+3. The confirm button reads exactly "Create".
+4. On save, a success toast reads exactly "Template created" and the new template appears in the list.</t>
         </is>
       </c>
       <c r="K82" s="15" t="inlineStr">
@@ -6809,13 +6809,13 @@
       <c r="I83" s="18" t="inlineStr">
         <is>
           <t>1. Click "New fee / discount".
-2. Set Type = "Discount"; Calculation type = "% of Subtotal"; Name = "ZZAUTOTEST Loyalty"; Percent = 8; Taxable = "No".
-3. Click "Add Fee / Discount".</t>
+2. Set Type = "Discount"; Calculation type = "% of Subtotal"; Name = "ZZAUTOTEST Loyalty"; Percent = 8; set the Taxable toggle OFF.
+3. Click "Create".</t>
         </is>
       </c>
       <c r="J83" s="18" t="inlineStr">
         <is>
-          <t>1. Save succeeds and the toast reads exactly "Discount added".
+          <t>1. Save succeeds and the toast reads exactly "Template created" (a generic message, not a per-type "Discount added").
 2. The template list shows "ZZAUTOTEST Loyalty", Type Discount, Calculation Type % of Subtotal, Amount −8%, Taxable No.</t>
         </is>
       </c>
@@ -6957,8 +6957,8 @@
       <c r="J85" s="18" t="inlineStr">
         <is>
           <t>1. Clicking the row opens the edit dialog titled "Edit Fee / Discount".
-2. The confirm button reads exactly "Save" (edit mode).
-3. On save, the toast reads exactly "Fee updated" and the list shows the new 7% value.</t>
+2. The confirm button reads exactly "Save" (edit mode); Type and Calculation type are locked (read-only) in template edit.
+3. On save, the toast reads exactly "Template updated" and the list shows the new 7% value.</t>
         </is>
       </c>
       <c r="K85" s="18" t="inlineStr">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="J87" s="18" t="inlineStr">
         <is>
-          <t>1. In addition to the standard message, the dialog adds exactly: "This template is set as a default for 2 customer(s). Their defaults will be removed too." (N reflects the actual number of customers).</t>
+          <t>1. In addition to the standard message, the dialog adds exactly: "This template is set as a default for 2 customer(s). Deleting it will remove it from them." (N reflects the actual number of customers).</t>
         </is>
       </c>
       <c r="K87" s="18" t="inlineStr">
@@ -8269,12 +8269,12 @@
       <c r="I104" s="15" t="inlineStr">
         <is>
           <t>1. Hover the Processing Fee entry in the WO Fees &amp; Discounts card and open its 3-dot menu.
-2. Attempt to remove it.</t>
+2. Note the available actions, then attempt to remove it.</t>
         </is>
       </c>
       <c r="J104" s="15" t="inlineStr">
         <is>
-          <t>1. The entry's menu offers "Delete" only — there is NO "Edit" for a Processing Fee.
+          <t>1. The entry's menu shows "Edit" and "Remove"; the Edit control is inert for a Processing Fee — attempting to edit it is rejected by the system (a Processing Fee cannot be edited on the WO instance).
 2. Removing it works normally (opens the "Remove Fee / Discount" confirm and removes on confirm).
 3. To change amount/method/taxable you must edit the TEMPLATE, not the WO instance.</t>
         </is>

</xml_diff>

<commit_message>
Fees & Discounts: fix audit findings (FD-CALC-018/019 plain-text, FD-WO-013 title, id-map titles)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
+++ b/build/fees-discounts/FeesDiscounts_V1_TestCases.xlsx
@@ -2012,7 +2012,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>Verify the whole-work-order Add Fee/Discount option is hidden without Work Orders: Create &amp; Edit</t>
+          <t>Verify the whole-work-order 'Add Work Order Fee / Discount' option is hidden without Work Orders: Create &amp; Edit</t>
         </is>
       </c>
       <c r="G14" s="20" t="inlineStr">
@@ -15055,8 +15055,8 @@
       </c>
       <c r="L176" s="15" t="inlineStr">
         <is>
-          <t>1. The Fees/Discounts row under Labor shows '↳ ttt' with a '+20%' badge and +$50.00.
-2. The part fee row shows '↳ test' with a '+11%' badge and +$2.20.
+          <t>1. The Fees/Discounts row under Labor shows '↳ ttt  +20%' and +$50.00 as plain text — no colored badge or pill.
+2. The part fee row shows '↳ test  +11%' and +$2.20 as plain text — no colored badge or pill.
 3. The collapsed line total at the top-right equals Labor + labor fee + Parts + part fee = $250.00 + $50.00 + $20.00 + $2.20 = $322.20.
 4. The line total is NOT $270.00 (it must not leave out the two fees).</t>
         </is>
@@ -15073,7 +15073,7 @@
       </c>
       <c r="O176" s="15" t="inlineStr">
         <is>
-          <t>SV-8480 (Story Defect under SV-8279, Epic SV-7387; PO Chris Ward): the per-line total_cost previously summed Labor + Parts gross only and ignored the line's own fees/discounts (showed $270.00). Fixed backend (Stefan Vukovic, PR ShopView/shopview#2228) to add the line's signed fee/discount amounts on top per spec S3-R18. Display-only, no stored values change. QA Passed on staging 2026-07-22. Concrete worked example from the ticket ($322.20) used as expected values.</t>
+          <t>SV-8480 (Story Defect under SV-8279, Epic SV-7387; PO Chris Ward): the per-line total_cost previously summed Labor + Parts gross only and ignored the line's own fees/discounts (showed $270.00). Fixed backend (Stefan Vukovic, PR ShopView/shopview#2228) to add the line's signed fee/discount amounts on top per spec S3-R18. Display-only, no stored values change. QA Passed on staging 2026-07-22. Concrete worked example from the ticket ($322.20) used as expected values. | SV-8479 item 4 de-badge 2026-07-22: line-level fee/discount rows reworded from '+20%'/'+11%' badge to PLAIN TEXT with the sign convention (no colored badge/pill), matching FD-INLINE-001/002; calc math ($322.20) unchanged.</t>
         </is>
       </c>
     </row>
@@ -15133,8 +15133,8 @@
       </c>
       <c r="L177" s="18" t="inlineStr">
         <is>
-          <t>1. The labor fee shows a '+20%' badge and a plus amount (+$50.00 on $250.00).
-2. The part discount shows a '-10%' badge and a minus amount (-$2.00 on $20.00).
+          <t>1. The labor fee shows '↳ &lt;name&gt;  +20%' and a plus amount (+$50.00 on $250.00) as plain text — no colored badge or pill.
+2. The part discount shows '↳ &lt;name&gt;  −10%' and a minus amount (−$2.00 on $20.00) as plain text — no colored badge or pill.
 3. The collapsed line total adds the fee and subtracts the discount: Labor $250.00 + fee $50.00 + Part $20.00 - discount $2.00 = $318.00.
 4. Fees increase the line total; discounts reduce it.</t>
         </is>
@@ -15151,7 +15151,7 @@
       </c>
       <c r="O177" s="18" t="inlineStr">
         <is>
-          <t>SV-8480 / S3-R18: the line total rolls in the line's SIGNED fee/discount amounts (fees add, discounts subtract). Complements FD-CALC-018 (all-fees case) by proving a discount subtracts.</t>
+          <t>SV-8480 / S3-R18: the line total rolls in the line's SIGNED fee/discount amounts (fees add, discounts subtract). Complements FD-CALC-018 (all-fees case) by proving a discount subtracts. | SV-8479 item 4 de-badge 2026-07-22: line-level fee/discount rows reworded from '+20%'/'-10%' badge to PLAIN TEXT with the sign convention (no colored badge/pill), matching FD-INLINE-001/002; calc math ($318.00) unchanged.</t>
         </is>
       </c>
     </row>
@@ -17787,7 +17787,7 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>Verify the whole-work-order Add Fee/Discount option is hidden without Work Orders: Create &amp; Edit</t>
+          <t>Verify the whole-work-order 'Add Work Order Fee / Discount' option is hidden without Work Orders: Create &amp; Edit</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">

</xml_diff>